<commit_message>
test: resultados de realizar los casos de prueba TC-V01, TC-C02 y TC-N03
</commit_message>
<xml_diff>
--- a/reportes/048_Casos_de_Prueba_Grupo7.xlsx
+++ b/reportes/048_Casos_de_Prueba_Grupo7.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javier Rivera\Documents\Proyecto IS\Proyecto QA - Grupo 7\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/56b5a6fa351e9256/Escritorio/PROYECTO_FINAL_CALIDAD/proyecto-qa-tienda/reportes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D91968F-DC6F-46E0-9941-872418632FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{1D91968F-DC6F-46E0-9941-872418632FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A344A76-9BC4-46FD-84AD-04E704253BBE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suite de pruebas" sheetId="1" r:id="rId1"/>
@@ -25,19 +25,14 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="181">
   <si>
     <t>OK</t>
   </si>
@@ -691,6 +686,15 @@
   </si>
   <si>
     <t xml:space="preserve">SUITE DE PRUEBAS - OPENCART DEMO (ABSTRACTA) · GRUPO 7 </t>
+  </si>
+  <si>
+    <t>Se mostró el mensaje "Thank you for your review. It has been submitted to the webmaster for approval." (traducción: "Gracias por tu reseña. Ha sido enviada al administrador para su aprobación.") y el formulario se limpió.</t>
+  </si>
+  <si>
+    <t>La reseña no se envió y se mostró "Warning: Review Text must be between 25 and 1000 characters!" (traducción: "Advertencia: el texto de la reseña debe tener entre 25 y 1000 caracteres").</t>
+  </si>
+  <si>
+    <t>No se envió el mensaje y aparecieron tres errores: "Name must be between 3 and 32 characters!" (el nombre debe tener entre 3 y 32 caracteres), "E-Mail Address does not appear to be valid!" (el correo electrónico no parece válido) y "Enquiry must be between 10 and 3000 characters!" (la consulta debe tener entre 10 y 3000 caracteres).</t>
   </si>
 </sst>
 </file>
@@ -700,7 +704,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,6 +755,13 @@
     </font>
     <font>
       <sz val="16"/>
+      <color theme="1"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Georgia"/>
       <family val="1"/>
@@ -809,7 +820,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -840,34 +851,25 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1170,45 +1172,64 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{FF775F78-5841-4D55-AEA5-1CD9581B8E64}">
+  <we:reference id="wa200010725" version="1.0.0.1" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200010725" version="1.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;51ea87f6-b902-4e7b-a058-bef645095cb2&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="29.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" style="3" customWidth="1"/>
     <col min="6" max="6" width="45" style="3" customWidth="1"/>
-    <col min="7" max="7" width="36.28515625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="38.7109375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="36.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="38.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" style="3" customWidth="1"/>
     <col min="10" max="10" width="14" style="3" customWidth="1"/>
-    <col min="11" max="12" width="14" style="21"/>
-    <col min="13" max="16384" width="14" style="3"/>
+    <col min="11" max="16384" width="14" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="10" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:13" s="10" customFormat="1" ht="18" customHeight="1">
+      <c r="A1" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="18"/>
       <c r="M1" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="11" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="11" customFormat="1" ht="28.95" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
@@ -1239,740 +1260,697 @@
       <c r="J2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
       <c r="M2" s="11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="14" t="s">
+    <row r="3" spans="1:13" s="8" customFormat="1" ht="15.6">
+      <c r="A3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
       <c r="M3" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="8" customFormat="1" ht="270" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:13" s="8" customFormat="1" ht="156">
+      <c r="A4" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="17" t="s">
+      <c r="H4" s="15"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-    </row>
-    <row r="5" spans="1:13" s="8" customFormat="1" ht="135" x14ac:dyDescent="0.2">
-      <c r="A5" s="16" t="s">
+    </row>
+    <row r="5" spans="1:13" s="8" customFormat="1" ht="93.6">
+      <c r="A5" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="17"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="17" t="s">
+      <c r="H5" s="15"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-    </row>
-    <row r="6" spans="1:13" s="8" customFormat="1" ht="210" x14ac:dyDescent="0.2">
-      <c r="A6" s="16" t="s">
+    </row>
+    <row r="6" spans="1:13" s="8" customFormat="1" ht="124.8">
+      <c r="A6" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="17"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="17" t="s">
+      <c r="H6" s="15"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-    </row>
-    <row r="7" spans="1:13" s="8" customFormat="1" ht="225" x14ac:dyDescent="0.2">
-      <c r="A7" s="16" t="s">
+    </row>
+    <row r="7" spans="1:13" s="8" customFormat="1" ht="140.4">
+      <c r="A7" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="17"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="17" t="s">
+      <c r="H7" s="15"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-    </row>
-    <row r="8" spans="1:13" s="8" customFormat="1" ht="330" x14ac:dyDescent="0.2">
-      <c r="A8" s="16" t="s">
+    </row>
+    <row r="8" spans="1:13" s="8" customFormat="1" ht="187.2">
+      <c r="A8" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="17"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="17" t="s">
+      <c r="H8" s="15"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-    </row>
-    <row r="9" spans="1:13" s="8" customFormat="1" ht="285" x14ac:dyDescent="0.2">
-      <c r="A9" s="16" t="s">
+    </row>
+    <row r="9" spans="1:13" s="8" customFormat="1" ht="171.6">
+      <c r="A9" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="17" t="s">
+      <c r="H9" s="15"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-    </row>
-    <row r="10" spans="1:13" s="8" customFormat="1" ht="270" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
+    </row>
+    <row r="10" spans="1:13" s="8" customFormat="1" ht="156">
+      <c r="A10" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="17"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="17" t="s">
+      <c r="H10" s="15"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-    </row>
-    <row r="11" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
+    </row>
+    <row r="11" spans="1:13" s="8" customFormat="1" ht="15.6">
+      <c r="A11" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-    </row>
-    <row r="12" spans="1:13" s="8" customFormat="1" ht="120" x14ac:dyDescent="0.2">
-      <c r="A12" s="16" t="s">
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+    </row>
+    <row r="12" spans="1:13" s="8" customFormat="1" ht="78">
+      <c r="A12" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="17"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="17" t="s">
+      <c r="H12" s="15"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-    </row>
-    <row r="13" spans="1:13" s="8" customFormat="1" ht="180" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
+    </row>
+    <row r="13" spans="1:13" s="8" customFormat="1" ht="140.4">
+      <c r="A13" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="17"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="17" t="s">
+      <c r="H13" s="15"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-    </row>
-    <row r="14" spans="1:13" s="8" customFormat="1" ht="135" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+    </row>
+    <row r="14" spans="1:13" s="8" customFormat="1" ht="93.6">
+      <c r="A14" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="17"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="17" t="s">
+      <c r="H14" s="15"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-    </row>
-    <row r="15" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
+    </row>
+    <row r="15" spans="1:13" s="8" customFormat="1" ht="15.6">
+      <c r="A15" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-    </row>
-    <row r="16" spans="1:13" s="8" customFormat="1" ht="120" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+    </row>
+    <row r="16" spans="1:13" s="8" customFormat="1" ht="93.6">
+      <c r="A16" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="H16" s="17"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="17" t="s">
+      <c r="H16" s="15"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-    </row>
-    <row r="17" spans="1:12" s="8" customFormat="1" ht="75" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
+    </row>
+    <row r="17" spans="1:12" s="8" customFormat="1" ht="62.4">
+      <c r="A17" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="17" t="s">
+      <c r="H17" s="15"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-    </row>
-    <row r="18" spans="1:12" s="8" customFormat="1" ht="180" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
+    </row>
+    <row r="18" spans="1:12" s="8" customFormat="1" ht="124.8">
+      <c r="A18" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="G18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="17" t="s">
+      <c r="H18" s="15"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-    </row>
-    <row r="19" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+    </row>
+    <row r="19" spans="1:12" s="8" customFormat="1" ht="15.6">
+      <c r="A19" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-    </row>
-    <row r="20" spans="1:12" s="8" customFormat="1" ht="225" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+    </row>
+    <row r="20" spans="1:12" s="8" customFormat="1" ht="124.8">
+      <c r="A20" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="G20" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="17"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="17" t="s">
+      <c r="H20" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J20" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="K20" s="20"/>
-      <c r="L20" s="20"/>
-    </row>
-    <row r="21" spans="1:12" s="8" customFormat="1" ht="210" x14ac:dyDescent="0.2">
-      <c r="A21" s="16" t="s">
+    </row>
+    <row r="21" spans="1:12" s="8" customFormat="1" ht="109.2">
+      <c r="A21" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="G21" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="H21" s="17"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="17" t="s">
+      <c r="H21" s="15"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
-    </row>
-    <row r="22" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+    </row>
+    <row r="22" spans="1:12" s="8" customFormat="1" ht="15.6">
+      <c r="A22" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="20"/>
-      <c r="L22" s="20"/>
-    </row>
-    <row r="23" spans="1:12" s="8" customFormat="1" ht="195" x14ac:dyDescent="0.2">
-      <c r="A23" s="16" t="s">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+    </row>
+    <row r="23" spans="1:12" s="8" customFormat="1" ht="109.2">
+      <c r="A23" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="G23" s="17" t="s">
+      <c r="G23" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="H23" s="17"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="17" t="s">
+      <c r="H23" s="15"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-    </row>
-    <row r="24" spans="1:12" s="8" customFormat="1" ht="195" x14ac:dyDescent="0.2">
-      <c r="A24" s="16" t="s">
+    </row>
+    <row r="24" spans="1:12" s="8" customFormat="1" ht="124.8">
+      <c r="A24" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="H24" s="17"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="17" t="s">
+      <c r="H24" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J24" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
-    </row>
-    <row r="25" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
+    </row>
+    <row r="25" spans="1:12" s="8" customFormat="1" ht="15.6">
+      <c r="A25" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
-    </row>
-    <row r="26" spans="1:12" s="8" customFormat="1" ht="180" x14ac:dyDescent="0.2">
-      <c r="A26" s="16" t="s">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+    </row>
+    <row r="26" spans="1:12" s="8" customFormat="1" ht="109.2">
+      <c r="A26" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="H26" s="17"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="17" t="s">
+      <c r="H26" s="15"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="K26" s="20"/>
-      <c r="L26" s="20"/>
-    </row>
-    <row r="27" spans="1:12" s="8" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A27" s="16" t="s">
+    </row>
+    <row r="27" spans="1:12" s="8" customFormat="1" ht="78">
+      <c r="A27" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="H27" s="17"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="17" t="s">
+      <c r="H27" s="15"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="K27" s="20"/>
       <c r="L27" s="20"/>
     </row>
-    <row r="28" spans="1:12" s="8" customFormat="1" ht="120" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
+    <row r="28" spans="1:12" s="8" customFormat="1" ht="156">
+      <c r="A28" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="H28" s="17"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="17" t="s">
+      <c r="H28" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="J28" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-    </row>
-    <row r="29" spans="1:12" s="8" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
+    </row>
+    <row r="29" spans="1:12" s="8" customFormat="1" ht="62.4">
+      <c r="A29" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="H29" s="17"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="17" t="s">
+      <c r="H29" s="15"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="K29" s="20"/>
-      <c r="L29" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2008,18 +1986,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="6" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="17.399999999999999">
       <c r="A1" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>157</v>
       </c>
@@ -2039,7 +2017,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>160</v>
       </c>
@@ -2064,7 +2042,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>161</v>
       </c>
@@ -2089,7 +2067,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>162</v>
       </c>
@@ -2114,7 +2092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>163</v>
       </c>
@@ -2124,7 +2102,7 @@
       </c>
       <c r="C7">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-V*",'Suite de pruebas'!$I:$I,"OK")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-V*",'Suite de pruebas'!$I:$I,"FALLO")</f>
@@ -2136,10 +2114,10 @@
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>164</v>
       </c>
@@ -2149,7 +2127,7 @@
       </c>
       <c r="C8">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-C*",'Suite de pruebas'!$I:$I,"OK")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-C*",'Suite de pruebas'!$I:$I,"FALLO")</f>
@@ -2161,10 +2139,10 @@
       </c>
       <c r="F8">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>165</v>
       </c>
@@ -2174,7 +2152,7 @@
       </c>
       <c r="C9">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-N*",'Suite de pruebas'!$I:$I,"OK")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9">
         <f>COUNTIFS('Suite de pruebas'!$A:$A,"TC-N*",'Suite de pruebas'!$I:$I,"FALLO")</f>
@@ -2186,10 +2164,10 @@
       </c>
       <c r="F9">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="5" t="s">
         <v>166</v>
       </c>
@@ -2199,7 +2177,7 @@
       </c>
       <c r="C10" s="5">
         <f>SUM(C4:C9)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="5">
         <f>SUM(D4:D9)</f>
@@ -2211,63 +2189,63 @@
       </c>
       <c r="F10" s="5">
         <f>SUM(F4:F9)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="5" t="s">
         <v>167</v>
       </c>
       <c r="B12" s="6">
         <f>IF(B10=0,0,(C10+D10+E10)/B10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0.14285714285714285</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="5" t="s">
         <v>168</v>
       </c>
       <c r="B13" s="6">
         <f>IF((C10+D10+E10)=0,0,C10/(C10+D10+E10))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1">
       <c r="A17" s="7" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1">
       <c r="A18" s="7" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1">
       <c r="A19" s="7" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1">
       <c r="A20" s="7" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1">
       <c r="A21" s="7" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1">
       <c r="A22" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1">
       <c r="A23" s="7" t="s">
         <v>176</v>
       </c>

</xml_diff>

<commit_message>
docs: capturas de evidencia en los casos ejecutados del Excel
</commit_message>
<xml_diff>
--- a/reportes/048_Casos_de_Prueba_Grupo7.xlsx
+++ b/reportes/048_Casos_de_Prueba_Grupo7.xlsx
@@ -179,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -233,6 +233,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,6 +333,161 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>3</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1600200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>8</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1609725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>12</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1609725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>19</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1524000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>23</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1514475"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>27</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1524000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -611,7 +769,7 @@
     <col width="36.33203125" customWidth="1" style="3" min="7" max="7"/>
     <col width="38.6640625" customWidth="1" style="3" min="8" max="8"/>
     <col width="19.109375" customWidth="1" style="3" min="9" max="9"/>
-    <col width="14" customWidth="1" style="3" min="10" max="10"/>
+    <col width="45" customWidth="1" style="3" min="10" max="10"/>
     <col width="14" customWidth="1" style="3" min="11" max="16384"/>
   </cols>
   <sheetData>
@@ -773,7 +931,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J4" s="23" t="inlineStr">
         <is>
           <t>TC-R01.png</t>
         </is>
@@ -1041,7 +1199,7 @@
           <t>FALLO</t>
         </is>
       </c>
-      <c r="J9" s="15" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>TC-R06.png</t>
         </is>
@@ -1165,7 +1323,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="140.4" customFormat="1" customHeight="1" s="8">
+    <row r="13" ht="152.25" customFormat="1" customHeight="1" s="8">
       <c r="A13" s="14" t="inlineStr">
         <is>
           <t>TC-L02</t>
@@ -1216,7 +1374,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="J13" s="15" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>TC-L02.png</t>
         </is>
@@ -1445,7 +1603,7 @@
       <c r="I19" s="21" t="n"/>
       <c r="J19" s="22" t="n"/>
     </row>
-    <row r="20" ht="124.8" customFormat="1" customHeight="1" s="8">
+    <row r="20" ht="145.5" customFormat="1" customHeight="1" s="8">
       <c r="A20" s="14" t="inlineStr">
         <is>
           <t>TC-V01</t>
@@ -1499,7 +1657,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="J20" s="15" t="inlineStr">
+      <c r="J20" s="23" t="inlineStr">
         <is>
           <t>TC-V01.png</t>
         </is>
@@ -1623,7 +1781,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="124.8" customFormat="1" customHeight="1" s="8">
+    <row r="24" ht="144.75" customFormat="1" customHeight="1" s="8">
       <c r="A24" s="14" t="inlineStr">
         <is>
           <t>TC-C02</t>
@@ -1676,7 +1834,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="J24" s="15" t="inlineStr">
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>TC-C02.png</t>
         </is>
@@ -1842,7 +2000,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="J28" s="15" t="inlineStr">
+      <c r="J28" s="23" t="inlineStr">
         <is>
           <t>TC-N03.png</t>
         </is>
@@ -1922,6 +2080,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
test: ejecución de los 15 casos restantes con capturas de evidencia
</commit_message>
<xml_diff>
--- a/reportes/048_Casos_de_Prueba_Grupo7.xlsx
+++ b/reportes/048_Casos_de_Prueba_Grupo7.xlsx
@@ -366,10 +366,10 @@
     <from>
       <col>9</col>
       <colOff>76200</colOff>
-      <row>8</row>
+      <row>4</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="2857500" cy="1609725"/>
+    <ext cx="2857500" cy="1790700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -391,10 +391,10 @@
     <from>
       <col>9</col>
       <colOff>76200</colOff>
-      <row>12</row>
+      <row>5</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="2857500" cy="1609725"/>
+    <ext cx="2857500" cy="1790700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -416,10 +416,10 @@
     <from>
       <col>9</col>
       <colOff>76200</colOff>
-      <row>19</row>
+      <row>6</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="2857500" cy="1524000"/>
+    <ext cx="2857500" cy="1790700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -441,10 +441,10 @@
     <from>
       <col>9</col>
       <colOff>76200</colOff>
-      <row>23</row>
+      <row>7</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="2857500" cy="1514475"/>
+    <ext cx="2838450" cy="3238500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -466,10 +466,10 @@
     <from>
       <col>9</col>
       <colOff>76200</colOff>
-      <row>27</row>
+      <row>8</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="2857500" cy="1524000"/>
+    <ext cx="2857500" cy="1609725"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -477,6 +477,381 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>9</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>11</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>12</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1609725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>13</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2838450" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>15</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2838450" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>16</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>17</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="1885950" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>19</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1524000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>20</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>22</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>23</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1514475"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>25</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2457450" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>26</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>27</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1524000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>76200</colOff>
+      <row>28</row>
+      <rowOff>228600</rowOff>
+    </from>
+    <ext cx="2857500" cy="1790700"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -937,7 +1312,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="93.59999999999999" customFormat="1" customHeight="1" s="8">
+    <row r="5" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>TC-R02</t>
@@ -978,15 +1353,23 @@
           <t>No se crea la cuenta y se muestra un mensaje de error debajo de cada campo obligatorio: First Name, Last Name, E-Mail, Telephone y Password.</t>
         </is>
       </c>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="14" t="n"/>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>No se creó la cuenta y se mostró un error debajo de cada campo obligatorio: "First Name must be between 1 and 32 characters!", "Last Name must be between 1 and 32 characters!", "E-Mail Address does not appear to be valid!", "Telephone must be between 3 and 32 characters!" y "Password must be between 4 and 20 characters!".</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr">
         <is>
           <t>TC-R02.png</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="124.8" customFormat="1" customHeight="1" s="8">
+    <row r="6" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>TC-R03</t>
@@ -1031,15 +1414,23 @@
           <t>No se crea la cuenta y se muestra el mensaje "Password confirmation does not match password!" debajo de "Password Confirm".</t>
         </is>
       </c>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="14" t="n"/>
-      <c r="J6" s="15" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>No se creó la cuenta y se mostró "Password confirmation does not match password!" debajo de "Password Confirm".</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr">
         <is>
           <t>TC-R03.png</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="140.4" customFormat="1" customHeight="1" s="8">
+    <row r="7" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>TC-R04</t>
@@ -1084,15 +1475,23 @@
           <t>No se crea una segunda cuenta y se muestra el mensaje "Warning: E-Mail Address is already registered!".</t>
         </is>
       </c>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="14" t="n"/>
-      <c r="J7" s="15" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>No se creó una segunda cuenta y se mostró "Warning: E-Mail Address is already registered!".</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr">
         <is>
           <t>TC-R04.png</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="187.2" customFormat="1" customHeight="1" s="8">
+    <row r="8" ht="280.5" customFormat="1" customHeight="1" s="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
           <t>TC-R05</t>
@@ -1136,9 +1535,17 @@
           <t>Con 32 caracteres, First Name no muestra error (solo aparece el de la confirmación). Con 33 caracteres se muestra "First Name must be between 1 and 32 characters!".</t>
         </is>
       </c>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="15" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Con 32 caracteres, First Name no mostró error (solo apareció el de la confirmación de contraseña). Con 33 caracteres se mostró "First Name must be between 1 and 32 characters!".</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>TC-R05.png</t>
         </is>
@@ -1205,7 +1612,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="156" customFormat="1" customHeight="1" s="8">
+    <row r="10" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A10" s="14" t="inlineStr">
         <is>
           <t>TC-R07</t>
@@ -1250,9 +1657,17 @@
           <t>Se muestra un mensaje en Password indicando los requisitos mínimos de seguridad (longitud y combinación de letras y números).</t>
         </is>
       </c>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="14" t="n"/>
-      <c r="J10" s="15" t="inlineStr">
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Password no mostró ningún error con "1234"; solo apareció "Password confirmation does not match password!". El sistema acepta contraseñas de 4 dígitos sin requisitos de seguridad. Corresponde al defecto DR-003.</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>FALLO</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>TC-R07.png</t>
         </is>
@@ -1274,7 +1689,7 @@
       <c r="I11" s="21" t="n"/>
       <c r="J11" s="22" t="n"/>
     </row>
-    <row r="12" ht="78" customFormat="1" customHeight="1" s="8">
+    <row r="12" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>TC-L01</t>
@@ -1315,9 +1730,17 @@
           <t>Se redirige a la página "My Account" con las opciones de la cuenta (Edit Account, Password, etc.).</t>
         </is>
       </c>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="14" t="n"/>
-      <c r="J12" s="15" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Se inició sesión y se redirigió a "My Account", con las opciones Edit Account, Password, Address Book y Wish List.</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>TC-L01.png</t>
         </is>
@@ -1380,7 +1803,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="93.59999999999999" customFormat="1" customHeight="1" s="8">
+    <row r="14" ht="280.5" customFormat="1" customHeight="1" s="8">
       <c r="A14" s="14" t="inlineStr">
         <is>
           <t>TC-L03</t>
@@ -1418,9 +1841,17 @@
           <t>Se muestra la página "Account Logout". Al intentar entrar a "My Account" después de cerrar sesión, el sitio redirige a la página de Login.</t>
         </is>
       </c>
-      <c r="H14" s="15" t="n"/>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="15" t="inlineStr">
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Se mostró la página de cierre de sesión (título "Account", ruta Account &gt; Logout) con el mensaje "You have been logged off your account". Al abrir "My Account" después de cerrar sesión, el sitio redirigió a la página de Login.</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>TC-L03.png</t>
         </is>
@@ -1442,7 +1873,7 @@
       <c r="I15" s="21" t="n"/>
       <c r="J15" s="22" t="n"/>
     </row>
-    <row r="16" ht="93.59999999999999" customFormat="1" customHeight="1" s="8">
+    <row r="16" ht="280.5" customFormat="1" customHeight="1" s="8">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t>TC-P01</t>
@@ -1481,15 +1912,23 @@
           <t>Se muestra "Success: Your account has been successfully updated." y al volver a "Edit Account" el teléfono es 55559876.</t>
         </is>
       </c>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="14" t="n"/>
-      <c r="J16" s="15" t="inlineStr">
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Se mostró "Success: Your account has been successfully updated." y, al volver a "Edit Account", el teléfono guardado era 55559876.</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>TC-P01.png</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="62.4" customFormat="1" customHeight="1" s="8">
+    <row r="17" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t>TC-P02</t>
@@ -1527,15 +1966,23 @@
           <t>No se guardan los cambios y se muestra "First Name must be between 1 and 32 characters!" debajo del campo.</t>
         </is>
       </c>
-      <c r="H17" s="15" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="15" t="inlineStr">
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>No se guardaron los cambios y se mostró "First Name must be between 1 and 32 characters!" debajo del campo. Al volver a "Edit Account", el nombre seguía siendo "Javier".</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>TC-P02.png</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="124.8" customFormat="1" customHeight="1" s="8">
+    <row r="18" ht="280.5" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="14" t="inlineStr">
         <is>
           <t>TC-P03</t>
@@ -1579,9 +2026,17 @@
           <t>Se muestra "Success: Your password has been successfully updated.". La contraseña anterior es rechazada y la nueva permite entrar a "My Account".</t>
         </is>
       </c>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="14" t="n"/>
-      <c r="J18" s="15" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>Se mostró "Success: Your password has been successfully updated.". Después de cerrar sesión, la contraseña anterior fue rechazada ("Warning: No match for E-Mail Address and/or Password.") y la nueva permitió entrar a "My Account".</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>TC-P03.png</t>
         </is>
@@ -1663,7 +2118,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="109.2" customFormat="1" customHeight="1" s="8">
+    <row r="21" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A21" s="14" t="inlineStr">
         <is>
           <t>TC-V02</t>
@@ -1706,9 +2161,17 @@
           <t>La reseña no se envía y se muestra el mensaje "Warning: Please select a review rating!".</t>
         </is>
       </c>
-      <c r="H21" s="15" t="n"/>
-      <c r="I21" s="14" t="n"/>
-      <c r="J21" s="15" t="inlineStr">
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>La reseña no se envió y se mostró "Warning: Please select a review rating!".</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J21" s="23" t="inlineStr">
         <is>
           <t>TC-V02.png</t>
         </is>
@@ -1730,7 +2193,7 @@
       <c r="I22" s="21" t="n"/>
       <c r="J22" s="22" t="n"/>
     </row>
-    <row r="23" ht="109.2" customFormat="1" customHeight="1" s="8">
+    <row r="23" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A23" s="14" t="inlineStr">
         <is>
           <t>TC-C01</t>
@@ -1773,9 +2236,17 @@
           <t>Se muestra el mensaje de confirmación "Thank you for your review. It has been submitted to the webmaster for approval.".</t>
         </is>
       </c>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="14" t="n"/>
-      <c r="J23" s="15" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Se mostró "Thank you for your review. It has been submitted to the webmaster for approval.".</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J23" s="23" t="inlineStr">
         <is>
           <t>TC-C01.png</t>
         </is>
@@ -1856,7 +2327,7 @@
       <c r="I25" s="21" t="n"/>
       <c r="J25" s="22" t="n"/>
     </row>
-    <row r="26" ht="109.2" customFormat="1" customHeight="1" s="8">
+    <row r="26" ht="280.5" customFormat="1" customHeight="1" s="8">
       <c r="A26" s="14" t="inlineStr">
         <is>
           <t>TC-N01</t>
@@ -1894,15 +2365,23 @@
           <t>Todas las categorías cargan sin errores visibles y el contador del menú lateral coincide con la cantidad de productos listados.</t>
         </is>
       </c>
-      <c r="H26" s="15" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="15" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Las 8 categorías cargaron sin errores visibles. En 6 el contador coincide con el listado, pero en Desktops el menú dice 13 y se listan 12 ("Showing 1 to 12 of 12"), y en Components el menú dice 2 y no se lista ningún producto. Corresponde al defecto DR-005.</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>FALLO</t>
+        </is>
+      </c>
+      <c r="J26" s="23" t="inlineStr">
         <is>
           <t>TC-N01.png</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="78" customFormat="1" customHeight="1" s="8">
+    <row r="27" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A27" s="14" t="inlineStr">
         <is>
           <t>TC-N02</t>
@@ -1940,9 +2419,17 @@
           <t>La página "Search - iPhone" muestra el producto iPhone y todos los resultados contienen "iPhone" en el nombre o la descripción.</t>
         </is>
       </c>
-      <c r="H27" s="15" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="15" t="inlineStr">
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Se mostró la página "Search - iPhone" con un único resultado: el producto iPhone.</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J27" s="23" t="inlineStr">
         <is>
           <t>TC-N02.png</t>
         </is>
@@ -2006,7 +2493,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="62.4" customFormat="1" customHeight="1" s="8">
+    <row r="29" ht="166.5" customFormat="1" customHeight="1" s="8">
       <c r="A29" s="14" t="inlineStr">
         <is>
           <t>TC-N04</t>
@@ -2044,9 +2531,17 @@
           <t>El sistema trata "%" como texto y muestra "There is no product that matches the search criteria.", sin errores.</t>
         </is>
       </c>
-      <c r="H29" s="15" t="n"/>
-      <c r="I29" s="14" t="n"/>
-      <c r="J29" s="15" t="inlineStr">
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>Se mostraron los 19 productos del catálogo ("Showing 1 to 15 of 19 (2 Pages)") en lugar del mensaje de que no hay resultados. El "%" se interpreta como comodín. Corresponde al defecto DR-001.</t>
+        </is>
+      </c>
+      <c r="I29" s="14" t="inlineStr">
+        <is>
+          <t>FALLO</t>
+        </is>
+      </c>
+      <c r="J29" s="23" t="inlineStr">
         <is>
           <t>TC-N04.png</t>
         </is>

</xml_diff>